<commit_message>
1.Fix errors in V02 MD files and tables 2.Update uhd two port read timing waveform 3.Modify PVT tables maxcolwidth in offdoc.py
</commit_message>
<xml_diff>
--- a/Template/SC/V02/Table/High Density Via Rom Compiler/Local_Datasheet_Config.xlsx
+++ b/Template/SC/V02/Table/High Density Via Rom Compiler/Local_Datasheet_Config.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22110" windowHeight="12300" activeTab="1"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="Table11" sheetId="21" r:id="rId1"/>
@@ -56,9 +56,7 @@
     <t>Default</t>
   </si>
   <si>
-    <t xml:space="preserve">LS (Light Sleep) - Control the WL driver source biasing to reduce static power. \
-Active high. The output state remains unchanged.
-</t>
+    <t>LS (Light Sleep) - Provides leakage reduction via fine-grained power gating and source biasing. Data Retention is valid for voltages above Vnom-10%.</t>
   </si>
   <si>
     <t>Enabled</t>
@@ -67,10 +65,8 @@
     <t>Advanced</t>
   </si>
   <si>
-    <t xml:space="preserve">LS (Light Sleep) - Control the WL driver source biasing.\
-DS (Deep Sleep) - Control the periphery circuit power gating, bitcell array hold the original data and memory outputs remain Logic Low.\
-SD (Shut Down) - Control the periphery circuit and bitcell array power gating, it performs a complete shutdown, bitcell array lose original data, and memory outputs remain Logic Low.
-</t>
+    <t>LS (Light Sleep) - Provides leakage reduction via fine-grained power gating and source biasing. Data Retention is valid for voltages above Vnom-10%. \
+SD (Shut Down) - When the SD pin is set high, performs a complete shutdown (power gating is applied to both the periphery and the array), with  data retention, and memory outputs remain Logic Low.</t>
   </si>
   <si>
     <t>Feature</t>
@@ -261,7 +257,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -314,13 +310,6 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
@@ -952,137 +941,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1159,22 +1148,19 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1509,39 +1495,39 @@
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="40.5" spans="1:4">
+    <row r="2" ht="27" spans="1:4">
       <c r="A2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="30" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="67.5" spans="1:4">
+    <row r="3" ht="54" spans="1:4">
       <c r="A3" s="23"/>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="30" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1567,24 +1553,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" spans="1:3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="27" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" ht="54.75" spans="1:3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="29" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>